<commit_message>
Refactor - enhanced glycosylation scanning logic
</commit_message>
<xml_diff>
--- a/tabular/refseq-lineage/ifnl-curated-side-data-mammalia-b.xlsx
+++ b/tabular/refseq-lineage/ifnl-curated-side-data-mammalia-b.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
   <workbookPr date1904="1" showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertgifford/Projects/host/IFNL-Evolution/tabular/refseq-lineage/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/rob/Projects/host/IFNL-Evolution/tabular/refseq-lineage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F75722A2-CC80-284C-961F-6978BCF893BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45093ABB-1309-C54F-B384-DB42E0AC4AAC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5780" yWindow="1200" windowWidth="33480" windowHeight="25340" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="900" yWindow="500" windowWidth="27900" windowHeight="17500" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IFNL-B" sheetId="2" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2613" uniqueCount="623">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2613" uniqueCount="622">
   <si>
     <t>retroIFNL1a</t>
   </si>
@@ -1688,12 +1688,6 @@
     <t>gene_clade</t>
   </si>
   <si>
-    <t>new group name</t>
-  </si>
-  <si>
-    <t>new subgroup name</t>
-  </si>
-  <si>
     <t>ND1</t>
   </si>
   <si>
@@ -1778,12 +1772,6 @@
     <t>Tubulidentata-16</t>
   </si>
   <si>
-    <t>new group name.new subgroup name</t>
-  </si>
-  <si>
-    <t>exon3456-new group name.new subgroup name</t>
-  </si>
-  <si>
     <t>Haplorhine-1.1</t>
   </si>
   <si>
@@ -1905,6 +1893,15 @@
   </si>
   <si>
     <t>Placental2_Scandentia-ND1</t>
+  </si>
+  <si>
+    <t>new group-subgroup name</t>
+  </si>
+  <si>
+    <t>ifnlb_exon3456_group</t>
+  </si>
+  <si>
+    <t>ifnlb_exon3456_subgroup</t>
   </si>
 </sst>
 </file>
@@ -2638,7 +2635,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2739,6 +2736,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="529">
@@ -3625,10 +3634,12 @@
     <col min="3" max="3" width="18.83203125" style="37" customWidth="1"/>
     <col min="4" max="4" width="28.6640625" style="37" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="7" width="17.83203125" customWidth="1"/>
-    <col min="8" max="9" width="25" customWidth="1"/>
-    <col min="10" max="10" width="16.1640625" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="17.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" customWidth="1"/>
+    <col min="8" max="8" width="13.1640625" customWidth="1"/>
+    <col min="9" max="9" width="25" style="37" customWidth="1"/>
+    <col min="10" max="10" width="16.1640625" style="37" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" style="37" customWidth="1"/>
     <col min="12" max="12" width="34.6640625" customWidth="1"/>
     <col min="13" max="13" width="21.83203125" customWidth="1"/>
     <col min="14" max="14" width="18" customWidth="1"/>
@@ -3653,25 +3664,25 @@
         <v>267</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>591</v>
+        <v>587</v>
       </c>
       <c r="F1" s="18" t="s">
         <v>486</v>
       </c>
       <c r="G1" s="18" t="s">
-        <v>581</v>
+        <v>487</v>
       </c>
       <c r="H1" s="18" t="s">
         <v>487</v>
       </c>
-      <c r="I1" s="18" t="s">
-        <v>580</v>
-      </c>
-      <c r="J1" s="18" t="s">
-        <v>550</v>
-      </c>
-      <c r="K1" s="18" t="s">
-        <v>551</v>
+      <c r="I1" s="35" t="s">
+        <v>619</v>
+      </c>
+      <c r="J1" s="35" t="s">
+        <v>620</v>
+      </c>
+      <c r="K1" s="35" t="s">
+        <v>621</v>
       </c>
       <c r="L1" s="18" t="s">
         <v>264</v>
@@ -3709,7 +3720,7 @@
         <v>246</v>
       </c>
       <c r="D2" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E2" s="23" t="s">
         <v>504</v>
@@ -3718,18 +3729,18 @@
         <v>501</v>
       </c>
       <c r="G2" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H2" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I2" s="23">
+        <v>553</v>
+      </c>
+      <c r="I2" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J2" s="23">
+      <c r="J2" s="34">
         <v>1</v>
       </c>
-      <c r="K2" s="23">
+      <c r="K2" s="34">
         <v>2</v>
       </c>
       <c r="L2" s="23" t="s">
@@ -3764,7 +3775,7 @@
         <v>246</v>
       </c>
       <c r="D3" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E3" s="23" t="s">
         <v>504</v>
@@ -3773,18 +3784,18 @@
         <v>501</v>
       </c>
       <c r="G3" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H3" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I3" s="23">
+        <v>553</v>
+      </c>
+      <c r="I3" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J3" s="23">
+      <c r="J3" s="34">
         <v>1</v>
       </c>
-      <c r="K3" s="23">
+      <c r="K3" s="34">
         <v>1</v>
       </c>
       <c r="L3" s="23" t="s">
@@ -3819,7 +3830,7 @@
         <v>246</v>
       </c>
       <c r="D4" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E4" s="23" t="s">
         <v>504</v>
@@ -3828,18 +3839,18 @@
         <v>501</v>
       </c>
       <c r="G4" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H4" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I4" s="23">
+        <v>553</v>
+      </c>
+      <c r="I4" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J4" s="23">
+      <c r="J4" s="34">
         <v>1</v>
       </c>
-      <c r="K4" s="23">
+      <c r="K4" s="34">
         <v>1</v>
       </c>
       <c r="L4" s="23" t="s">
@@ -3878,7 +3889,7 @@
         <v>246</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E5" s="26" t="s">
         <v>504</v>
@@ -3887,18 +3898,18 @@
         <v>501</v>
       </c>
       <c r="G5" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H5" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I5" s="26">
+        <v>553</v>
+      </c>
+      <c r="I5" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J5" s="26">
+      <c r="J5" s="39">
         <v>1</v>
       </c>
-      <c r="K5" s="23">
+      <c r="K5" s="34">
         <v>1</v>
       </c>
       <c r="L5" s="26" t="s">
@@ -3931,7 +3942,7 @@
         <v>246</v>
       </c>
       <c r="D6" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E6" s="26" t="s">
         <v>504</v>
@@ -3940,18 +3951,18 @@
         <v>501</v>
       </c>
       <c r="G6" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H6" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I6" s="26">
+        <v>553</v>
+      </c>
+      <c r="I6" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J6" s="26">
+      <c r="J6" s="39">
         <v>1</v>
       </c>
-      <c r="K6" s="23">
+      <c r="K6" s="34">
         <v>1</v>
       </c>
       <c r="L6" s="26" t="s">
@@ -3984,7 +3995,7 @@
         <v>246</v>
       </c>
       <c r="D7" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E7" s="26" t="s">
         <v>504</v>
@@ -3993,18 +4004,18 @@
         <v>501</v>
       </c>
       <c r="G7" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H7" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I7" s="26">
+        <v>553</v>
+      </c>
+      <c r="I7" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J7" s="26">
+      <c r="J7" s="39">
         <v>1</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="34">
         <v>1</v>
       </c>
       <c r="L7" s="26" t="s">
@@ -4037,7 +4048,7 @@
         <v>246</v>
       </c>
       <c r="D8" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E8" s="26" t="s">
         <v>504</v>
@@ -4046,18 +4057,18 @@
         <v>501</v>
       </c>
       <c r="G8" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H8" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I8" s="26">
+        <v>553</v>
+      </c>
+      <c r="I8" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J8" s="26">
+      <c r="J8" s="39">
         <v>1</v>
       </c>
-      <c r="K8" s="23">
+      <c r="K8" s="34">
         <v>1</v>
       </c>
       <c r="L8" s="26" t="s">
@@ -4090,7 +4101,7 @@
         <v>246</v>
       </c>
       <c r="D9" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E9" s="26" t="s">
         <v>504</v>
@@ -4099,18 +4110,18 @@
         <v>501</v>
       </c>
       <c r="G9" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I9" s="26">
+        <v>553</v>
+      </c>
+      <c r="I9" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J9" s="26">
+      <c r="J9" s="39">
         <v>1</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="34">
         <v>1</v>
       </c>
       <c r="L9" s="26" t="s">
@@ -4143,7 +4154,7 @@
         <v>246</v>
       </c>
       <c r="D10" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E10" s="26" t="s">
         <v>504</v>
@@ -4152,18 +4163,18 @@
         <v>501</v>
       </c>
       <c r="G10" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H10" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I10" s="26">
+        <v>553</v>
+      </c>
+      <c r="I10" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J10" s="26">
+      <c r="J10" s="39">
         <v>1</v>
       </c>
-      <c r="K10" s="23">
+      <c r="K10" s="34">
         <v>1</v>
       </c>
       <c r="L10" s="26" t="s">
@@ -4196,7 +4207,7 @@
         <v>246</v>
       </c>
       <c r="D11" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E11" s="26" t="s">
         <v>504</v>
@@ -4205,18 +4216,18 @@
         <v>501</v>
       </c>
       <c r="G11" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H11" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I11" s="26">
+        <v>553</v>
+      </c>
+      <c r="I11" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J11" s="26">
+      <c r="J11" s="39">
         <v>1</v>
       </c>
-      <c r="K11" s="23">
+      <c r="K11" s="34">
         <v>1</v>
       </c>
       <c r="L11" s="26" t="s">
@@ -4249,7 +4260,7 @@
         <v>246</v>
       </c>
       <c r="D12" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E12" s="26" t="s">
         <v>504</v>
@@ -4258,18 +4269,18 @@
         <v>501</v>
       </c>
       <c r="G12" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H12" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I12" s="26">
+        <v>553</v>
+      </c>
+      <c r="I12" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J12" s="26">
+      <c r="J12" s="39">
         <v>1</v>
       </c>
-      <c r="K12" s="23">
+      <c r="K12" s="34">
         <v>1</v>
       </c>
       <c r="L12" s="26" t="s">
@@ -4302,7 +4313,7 @@
         <v>246</v>
       </c>
       <c r="D13" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E13" s="26" t="s">
         <v>504</v>
@@ -4311,18 +4322,18 @@
         <v>501</v>
       </c>
       <c r="G13" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H13" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I13" s="26">
+        <v>553</v>
+      </c>
+      <c r="I13" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J13" s="26">
+      <c r="J13" s="39">
         <v>1</v>
       </c>
-      <c r="K13" s="23">
+      <c r="K13" s="34">
         <v>1</v>
       </c>
       <c r="L13" s="26" t="s">
@@ -4355,7 +4366,7 @@
         <v>246</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E14" s="26" t="s">
         <v>504</v>
@@ -4364,18 +4375,18 @@
         <v>501</v>
       </c>
       <c r="G14" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H14" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I14" s="26">
+        <v>553</v>
+      </c>
+      <c r="I14" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J14" s="26">
+      <c r="J14" s="39">
         <v>1</v>
       </c>
-      <c r="K14" s="23">
+      <c r="K14" s="34">
         <v>2</v>
       </c>
       <c r="L14" s="26" t="s">
@@ -4408,7 +4419,7 @@
         <v>246</v>
       </c>
       <c r="D15" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>510</v>
@@ -4417,18 +4428,18 @@
         <v>500</v>
       </c>
       <c r="G15" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I15" s="23">
+        <v>553</v>
+      </c>
+      <c r="I15" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J15" s="23">
+      <c r="J15" s="34">
         <v>1</v>
       </c>
-      <c r="K15" s="23">
+      <c r="K15" s="34">
         <v>2</v>
       </c>
       <c r="L15" s="23" t="s">
@@ -4461,7 +4472,7 @@
         <v>246</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E16" s="23" t="s">
         <v>510</v>
@@ -4470,18 +4481,18 @@
         <v>500</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H16" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I16" s="23">
+        <v>553</v>
+      </c>
+      <c r="I16" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J16" s="23">
+      <c r="J16" s="34">
         <v>1</v>
       </c>
-      <c r="K16" s="23">
+      <c r="K16" s="34">
         <v>2</v>
       </c>
       <c r="L16" s="23" t="s">
@@ -4514,7 +4525,7 @@
         <v>246</v>
       </c>
       <c r="D17" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E17" s="23" t="s">
         <v>510</v>
@@ -4523,18 +4534,18 @@
         <v>500</v>
       </c>
       <c r="G17" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I17" s="23">
+        <v>553</v>
+      </c>
+      <c r="I17" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="34">
         <v>1</v>
       </c>
-      <c r="K17" s="23">
+      <c r="K17" s="34">
         <v>2</v>
       </c>
       <c r="L17" s="23" t="s">
@@ -4567,7 +4578,7 @@
         <v>246</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E18" s="23" t="s">
         <v>510</v>
@@ -4576,18 +4587,18 @@
         <v>500</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H18" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I18" s="23">
+        <v>553</v>
+      </c>
+      <c r="I18" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J18" s="23">
+      <c r="J18" s="34">
         <v>1</v>
       </c>
-      <c r="K18" s="23">
+      <c r="K18" s="34">
         <v>2</v>
       </c>
       <c r="L18" s="23" t="s">
@@ -4620,7 +4631,7 @@
         <v>246</v>
       </c>
       <c r="D19" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E19" s="23" t="s">
         <v>510</v>
@@ -4629,18 +4640,18 @@
         <v>500</v>
       </c>
       <c r="G19" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I19" s="23">
+        <v>553</v>
+      </c>
+      <c r="I19" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J19" s="23">
+      <c r="J19" s="34">
         <v>1</v>
       </c>
-      <c r="K19" s="23">
+      <c r="K19" s="34">
         <v>2</v>
       </c>
       <c r="L19" s="23" t="s">
@@ -4673,7 +4684,7 @@
         <v>246</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E20" s="23" t="s">
         <v>510</v>
@@ -4682,18 +4693,18 @@
         <v>500</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H20" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I20" s="23">
+        <v>553</v>
+      </c>
+      <c r="I20" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J20" s="23">
+      <c r="J20" s="34">
         <v>1</v>
       </c>
-      <c r="K20" s="23">
+      <c r="K20" s="34">
         <v>2</v>
       </c>
       <c r="L20" s="23" t="s">
@@ -4726,7 +4737,7 @@
         <v>246</v>
       </c>
       <c r="D21" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E21" s="23" t="s">
         <v>510</v>
@@ -4735,18 +4746,18 @@
         <v>500</v>
       </c>
       <c r="G21" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I21" s="23">
+        <v>553</v>
+      </c>
+      <c r="I21" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J21" s="23">
+      <c r="J21" s="34">
         <v>1</v>
       </c>
-      <c r="K21" s="23">
+      <c r="K21" s="34">
         <v>2</v>
       </c>
       <c r="L21" s="23" t="s">
@@ -4779,7 +4790,7 @@
         <v>246</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E22" s="23" t="s">
         <v>510</v>
@@ -4788,18 +4799,18 @@
         <v>500</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H22" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I22" s="23">
+        <v>553</v>
+      </c>
+      <c r="I22" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J22" s="23">
+      <c r="J22" s="34">
         <v>1</v>
       </c>
-      <c r="K22" s="23">
+      <c r="K22" s="34">
         <v>2</v>
       </c>
       <c r="L22" s="23" t="s">
@@ -4836,7 +4847,7 @@
         <v>246</v>
       </c>
       <c r="D23" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E23" s="23" t="s">
         <v>510</v>
@@ -4845,18 +4856,18 @@
         <v>500</v>
       </c>
       <c r="G23" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I23" s="23">
+        <v>553</v>
+      </c>
+      <c r="I23" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J23" s="23">
+      <c r="J23" s="34">
         <v>1</v>
       </c>
-      <c r="K23" s="23">
+      <c r="K23" s="34">
         <v>2</v>
       </c>
       <c r="L23" s="23" t="s">
@@ -4889,7 +4900,7 @@
         <v>246</v>
       </c>
       <c r="D24" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E24" s="23" t="s">
         <v>510</v>
@@ -4898,18 +4909,18 @@
         <v>500</v>
       </c>
       <c r="G24" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H24" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I24" s="23">
+        <v>553</v>
+      </c>
+      <c r="I24" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J24" s="23">
+      <c r="J24" s="34">
         <v>1</v>
       </c>
-      <c r="K24" s="23">
+      <c r="K24" s="34">
         <v>2</v>
       </c>
       <c r="L24" s="23" t="s">
@@ -4942,7 +4953,7 @@
         <v>246</v>
       </c>
       <c r="D25" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E25" s="23" t="s">
         <v>510</v>
@@ -4951,18 +4962,18 @@
         <v>500</v>
       </c>
       <c r="G25" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H25" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I25" s="23">
+        <v>553</v>
+      </c>
+      <c r="I25" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J25" s="23">
+      <c r="J25" s="34">
         <v>1</v>
       </c>
-      <c r="K25" s="23">
+      <c r="K25" s="34">
         <v>2</v>
       </c>
       <c r="L25" s="23" t="s">
@@ -4995,7 +5006,7 @@
         <v>246</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E26" s="23" t="s">
         <v>510</v>
@@ -5004,18 +5015,18 @@
         <v>500</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H26" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I26" s="23">
+        <v>553</v>
+      </c>
+      <c r="I26" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J26" s="23">
+      <c r="J26" s="34">
         <v>1</v>
       </c>
-      <c r="K26" s="23">
+      <c r="K26" s="34">
         <v>2</v>
       </c>
       <c r="L26" s="23" t="s">
@@ -5048,7 +5059,7 @@
         <v>246</v>
       </c>
       <c r="D27" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E27" s="23" t="s">
         <v>510</v>
@@ -5057,18 +5068,18 @@
         <v>500</v>
       </c>
       <c r="G27" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H27" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I27" s="23">
+        <v>553</v>
+      </c>
+      <c r="I27" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J27" s="23">
+      <c r="J27" s="34">
         <v>1</v>
       </c>
-      <c r="K27" s="23">
+      <c r="K27" s="34">
         <v>2</v>
       </c>
       <c r="L27" s="23" t="s">
@@ -5101,7 +5112,7 @@
         <v>246</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E28" s="23" t="s">
         <v>510</v>
@@ -5110,18 +5121,18 @@
         <v>500</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H28" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I28" s="23">
+        <v>553</v>
+      </c>
+      <c r="I28" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J28" s="23">
+      <c r="J28" s="34">
         <v>1</v>
       </c>
-      <c r="K28" s="23">
+      <c r="K28" s="34">
         <v>2</v>
       </c>
       <c r="L28" s="23" t="s">
@@ -5154,7 +5165,7 @@
         <v>246</v>
       </c>
       <c r="D29" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E29" s="23" t="s">
         <v>510</v>
@@ -5163,18 +5174,18 @@
         <v>500</v>
       </c>
       <c r="G29" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H29" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I29" s="23">
+        <v>553</v>
+      </c>
+      <c r="I29" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J29" s="23">
+      <c r="J29" s="34">
         <v>1</v>
       </c>
-      <c r="K29" s="23">
+      <c r="K29" s="34">
         <v>2</v>
       </c>
       <c r="L29" s="23" t="s">
@@ -5207,7 +5218,7 @@
         <v>246</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E30" s="23" t="s">
         <v>510</v>
@@ -5216,18 +5227,18 @@
         <v>500</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H30" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I30" s="23">
+        <v>553</v>
+      </c>
+      <c r="I30" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J30" s="23">
+      <c r="J30" s="34">
         <v>1</v>
       </c>
-      <c r="K30" s="23">
+      <c r="K30" s="34">
         <v>2</v>
       </c>
       <c r="L30" s="23" t="s">
@@ -5260,7 +5271,7 @@
         <v>246</v>
       </c>
       <c r="D31" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E31" s="23" t="s">
         <v>510</v>
@@ -5269,18 +5280,18 @@
         <v>500</v>
       </c>
       <c r="G31" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H31" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I31" s="23">
+        <v>553</v>
+      </c>
+      <c r="I31" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J31" s="23">
+      <c r="J31" s="34">
         <v>1</v>
       </c>
-      <c r="K31" s="23">
+      <c r="K31" s="34">
         <v>2</v>
       </c>
       <c r="L31" s="23" t="s">
@@ -5313,7 +5324,7 @@
         <v>246</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E32" s="23" t="s">
         <v>510</v>
@@ -5322,18 +5333,18 @@
         <v>500</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H32" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I32" s="23">
+        <v>553</v>
+      </c>
+      <c r="I32" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J32" s="23">
+      <c r="J32" s="34">
         <v>1</v>
       </c>
-      <c r="K32" s="23">
+      <c r="K32" s="34">
         <v>2</v>
       </c>
       <c r="L32" s="23" t="s">
@@ -5368,7 +5379,7 @@
         <v>246</v>
       </c>
       <c r="D33" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E33" s="23" t="s">
         <v>510</v>
@@ -5377,18 +5388,18 @@
         <v>500</v>
       </c>
       <c r="G33" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H33" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I33" s="23">
+        <v>553</v>
+      </c>
+      <c r="I33" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J33" s="23">
+      <c r="J33" s="34">
         <v>1</v>
       </c>
-      <c r="K33" s="23">
+      <c r="K33" s="34">
         <v>2</v>
       </c>
       <c r="L33" s="23" t="s">
@@ -5421,7 +5432,7 @@
         <v>246</v>
       </c>
       <c r="D34" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E34" s="23" t="s">
         <v>510</v>
@@ -5430,18 +5441,18 @@
         <v>500</v>
       </c>
       <c r="G34" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H34" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I34" s="23">
+        <v>553</v>
+      </c>
+      <c r="I34" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J34" s="23">
+      <c r="J34" s="34">
         <v>1</v>
       </c>
-      <c r="K34" s="23">
+      <c r="K34" s="34">
         <v>2</v>
       </c>
       <c r="L34" s="23" t="s">
@@ -5476,7 +5487,7 @@
         <v>246</v>
       </c>
       <c r="D35" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E35" s="23" t="s">
         <v>510</v>
@@ -5485,18 +5496,18 @@
         <v>500</v>
       </c>
       <c r="G35" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H35" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I35" s="23">
+        <v>553</v>
+      </c>
+      <c r="I35" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J35" s="23">
+      <c r="J35" s="34">
         <v>1</v>
       </c>
-      <c r="K35" s="23">
+      <c r="K35" s="34">
         <v>2</v>
       </c>
       <c r="L35" s="23" t="s">
@@ -5531,7 +5542,7 @@
         <v>246</v>
       </c>
       <c r="D36" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E36" s="23" t="s">
         <v>510</v>
@@ -5540,18 +5551,18 @@
         <v>500</v>
       </c>
       <c r="G36" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H36" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I36" s="23">
+        <v>553</v>
+      </c>
+      <c r="I36" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J36" s="23">
+      <c r="J36" s="34">
         <v>1</v>
       </c>
-      <c r="K36" s="23">
+      <c r="K36" s="34">
         <v>2</v>
       </c>
       <c r="L36" s="23" t="s">
@@ -5584,7 +5595,7 @@
         <v>246</v>
       </c>
       <c r="D37" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E37" s="23" t="s">
         <v>510</v>
@@ -5593,18 +5604,18 @@
         <v>500</v>
       </c>
       <c r="G37" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H37" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I37" s="23">
+        <v>553</v>
+      </c>
+      <c r="I37" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J37" s="23">
+      <c r="J37" s="34">
         <v>1</v>
       </c>
-      <c r="K37" s="23">
+      <c r="K37" s="34">
         <v>2</v>
       </c>
       <c r="L37" s="23" t="s">
@@ -5637,7 +5648,7 @@
         <v>246</v>
       </c>
       <c r="D38" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E38" s="23" t="s">
         <v>510</v>
@@ -5646,18 +5657,18 @@
         <v>500</v>
       </c>
       <c r="G38" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H38" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I38" s="23">
+        <v>553</v>
+      </c>
+      <c r="I38" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J38" s="23">
+      <c r="J38" s="34">
         <v>1</v>
       </c>
-      <c r="K38" s="23">
+      <c r="K38" s="34">
         <v>2</v>
       </c>
       <c r="L38" s="23" t="s">
@@ -5690,7 +5701,7 @@
         <v>246</v>
       </c>
       <c r="D39" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E39" s="26" t="s">
         <v>510</v>
@@ -5699,18 +5710,18 @@
         <v>500</v>
       </c>
       <c r="G39" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H39" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I39" s="26">
+        <v>553</v>
+      </c>
+      <c r="I39" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J39" s="26">
+      <c r="J39" s="39">
         <v>1</v>
       </c>
-      <c r="K39" s="23">
+      <c r="K39" s="34">
         <v>2</v>
       </c>
       <c r="L39" s="26" t="s">
@@ -5743,7 +5754,7 @@
         <v>246</v>
       </c>
       <c r="D40" s="23" t="s">
-        <v>593</v>
+        <v>589</v>
       </c>
       <c r="E40" s="26" t="s">
         <v>510</v>
@@ -5752,18 +5763,18 @@
         <v>500</v>
       </c>
       <c r="G40" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H40" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I40" s="26">
+        <v>553</v>
+      </c>
+      <c r="I40" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J40" s="26">
+      <c r="J40" s="39">
         <v>1</v>
       </c>
-      <c r="K40" s="23">
+      <c r="K40" s="34">
         <v>2</v>
       </c>
       <c r="L40" s="26" t="s">
@@ -5796,7 +5807,7 @@
         <v>246</v>
       </c>
       <c r="D41" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E41" s="23" t="s">
         <v>504</v>
@@ -5805,18 +5816,18 @@
         <v>501</v>
       </c>
       <c r="G41" s="23" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H41" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I41" s="23">
+        <v>553</v>
+      </c>
+      <c r="I41" s="34">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J41" s="23">
+      <c r="J41" s="34">
         <v>1</v>
       </c>
-      <c r="K41" s="23">
+      <c r="K41" s="34">
         <v>2</v>
       </c>
       <c r="L41" s="23" t="s">
@@ -5851,7 +5862,7 @@
         <v>246</v>
       </c>
       <c r="D42" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E42" s="26" t="s">
         <v>504</v>
@@ -5860,18 +5871,18 @@
         <v>501</v>
       </c>
       <c r="G42" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H42" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I42" s="26">
+        <v>553</v>
+      </c>
+      <c r="I42" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J42" s="26">
+      <c r="J42" s="39">
         <v>1</v>
       </c>
-      <c r="K42" s="26">
+      <c r="K42" s="39">
         <v>2</v>
       </c>
       <c r="L42" s="26" t="s">
@@ -5904,7 +5915,7 @@
         <v>246</v>
       </c>
       <c r="D43" s="23" t="s">
-        <v>592</v>
+        <v>588</v>
       </c>
       <c r="E43" s="26" t="s">
         <v>504</v>
@@ -5913,18 +5924,18 @@
         <v>501</v>
       </c>
       <c r="G43" s="26" t="s">
-        <v>582</v>
+        <v>578</v>
       </c>
       <c r="H43" s="26" t="s">
-        <v>555</v>
-      </c>
-      <c r="I43" s="26">
+        <v>553</v>
+      </c>
+      <c r="I43" s="39">
         <v>1.1000000000000001</v>
       </c>
-      <c r="J43" s="26">
+      <c r="J43" s="39">
         <v>1</v>
       </c>
-      <c r="K43" s="26">
+      <c r="K43" s="39">
         <v>2</v>
       </c>
       <c r="L43" s="23" t="s">
@@ -5957,7 +5968,7 @@
         <v>246</v>
       </c>
       <c r="D44" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E44" s="23" t="s">
         <v>510</v>
@@ -5966,18 +5977,18 @@
         <v>500</v>
       </c>
       <c r="G44" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H44" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I44" s="23">
+        <v>553</v>
+      </c>
+      <c r="I44" s="34">
         <v>1.2</v>
       </c>
-      <c r="J44" s="23">
+      <c r="J44" s="34">
         <v>1</v>
       </c>
-      <c r="K44" s="23">
+      <c r="K44" s="34">
         <v>2</v>
       </c>
       <c r="L44" s="23" t="s">
@@ -6010,7 +6021,7 @@
         <v>246</v>
       </c>
       <c r="D45" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E45" s="23" t="s">
         <v>510</v>
@@ -6019,18 +6030,18 @@
         <v>500</v>
       </c>
       <c r="G45" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H45" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I45" s="23">
+        <v>553</v>
+      </c>
+      <c r="I45" s="34">
         <v>1.2</v>
       </c>
-      <c r="J45" s="23">
+      <c r="J45" s="34">
         <v>1</v>
       </c>
-      <c r="K45" s="23">
+      <c r="K45" s="34">
         <v>2</v>
       </c>
       <c r="L45" s="23" t="s">
@@ -6065,7 +6076,7 @@
         <v>246</v>
       </c>
       <c r="D46" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E46" s="23" t="s">
         <v>510</v>
@@ -6074,18 +6085,18 @@
         <v>500</v>
       </c>
       <c r="G46" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H46" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I46" s="23">
+        <v>553</v>
+      </c>
+      <c r="I46" s="34">
         <v>1.2</v>
       </c>
-      <c r="J46" s="23">
+      <c r="J46" s="34">
         <v>1</v>
       </c>
-      <c r="K46" s="23">
+      <c r="K46" s="34">
         <v>2</v>
       </c>
       <c r="L46" s="23" t="s">
@@ -6118,7 +6129,7 @@
         <v>246</v>
       </c>
       <c r="D47" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E47" s="23" t="s">
         <v>510</v>
@@ -6127,18 +6138,18 @@
         <v>500</v>
       </c>
       <c r="G47" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H47" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I47" s="23">
+        <v>553</v>
+      </c>
+      <c r="I47" s="34">
         <v>1.2</v>
       </c>
-      <c r="J47" s="23">
+      <c r="J47" s="34">
         <v>1</v>
       </c>
-      <c r="K47" s="23">
+      <c r="K47" s="34">
         <v>2</v>
       </c>
       <c r="L47" s="23" t="s">
@@ -6171,7 +6182,7 @@
         <v>246</v>
       </c>
       <c r="D48" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E48" s="23" t="s">
         <v>510</v>
@@ -6180,18 +6191,18 @@
         <v>500</v>
       </c>
       <c r="G48" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H48" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I48" s="23">
+        <v>553</v>
+      </c>
+      <c r="I48" s="34">
         <v>1.2</v>
       </c>
-      <c r="J48" s="23">
+      <c r="J48" s="34">
         <v>1</v>
       </c>
-      <c r="K48" s="23">
+      <c r="K48" s="34">
         <v>2</v>
       </c>
       <c r="L48" s="23" t="s">
@@ -6226,7 +6237,7 @@
         <v>246</v>
       </c>
       <c r="D49" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E49" s="23" t="s">
         <v>510</v>
@@ -6235,18 +6246,18 @@
         <v>500</v>
       </c>
       <c r="G49" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H49" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I49" s="23">
+        <v>553</v>
+      </c>
+      <c r="I49" s="34">
         <v>1.2</v>
       </c>
-      <c r="J49" s="23">
+      <c r="J49" s="34">
         <v>1</v>
       </c>
-      <c r="K49" s="23">
+      <c r="K49" s="34">
         <v>2</v>
       </c>
       <c r="L49" s="23" t="s">
@@ -6279,7 +6290,7 @@
         <v>246</v>
       </c>
       <c r="D50" s="23" t="s">
-        <v>594</v>
+        <v>590</v>
       </c>
       <c r="E50" s="23" t="s">
         <v>510</v>
@@ -6288,18 +6299,18 @@
         <v>500</v>
       </c>
       <c r="G50" s="23" t="s">
-        <v>583</v>
+        <v>579</v>
       </c>
       <c r="H50" s="23" t="s">
-        <v>555</v>
-      </c>
-      <c r="I50" s="23">
+        <v>553</v>
+      </c>
+      <c r="I50" s="34">
         <v>1.2</v>
       </c>
-      <c r="J50" s="23">
+      <c r="J50" s="34">
         <v>1</v>
       </c>
-      <c r="K50" s="23">
+      <c r="K50" s="34">
         <v>2</v>
       </c>
       <c r="L50" s="23" t="s">
@@ -6332,7 +6343,7 @@
         <v>246</v>
       </c>
       <c r="D51" s="23" t="s">
-        <v>595</v>
+        <v>591</v>
       </c>
       <c r="E51" s="23" t="s">
         <v>512</v>
@@ -6341,18 +6352,18 @@
         <v>499</v>
       </c>
       <c r="G51" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H51" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I51" s="23">
+        <v>554</v>
+      </c>
+      <c r="I51" s="34">
         <v>2.1</v>
       </c>
-      <c r="J51" s="23">
+      <c r="J51" s="34">
         <v>2</v>
       </c>
-      <c r="K51" s="23">
+      <c r="K51" s="34">
         <v>1</v>
       </c>
       <c r="L51" s="23" t="s">
@@ -6387,7 +6398,7 @@
         <v>246</v>
       </c>
       <c r="D52" s="23" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E52" s="23" t="s">
         <v>511</v>
@@ -6396,18 +6407,18 @@
         <v>500</v>
       </c>
       <c r="G52" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H52" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I52" s="23">
+        <v>554</v>
+      </c>
+      <c r="I52" s="34">
         <v>2.1</v>
       </c>
-      <c r="J52" s="23">
+      <c r="J52" s="34">
         <v>2</v>
       </c>
-      <c r="K52" s="23">
+      <c r="K52" s="34">
         <v>1</v>
       </c>
       <c r="L52" s="23" t="s">
@@ -6442,7 +6453,7 @@
         <v>246</v>
       </c>
       <c r="D53" s="23" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E53" s="23" t="s">
         <v>511</v>
@@ -6451,18 +6462,18 @@
         <v>500</v>
       </c>
       <c r="G53" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H53" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I53" s="23">
+        <v>554</v>
+      </c>
+      <c r="I53" s="34">
         <v>2.1</v>
       </c>
-      <c r="J53" s="23">
+      <c r="J53" s="34">
         <v>2</v>
       </c>
-      <c r="K53" s="23">
+      <c r="K53" s="34">
         <v>1</v>
       </c>
       <c r="L53" s="23" t="s">
@@ -6497,7 +6508,7 @@
         <v>246</v>
       </c>
       <c r="D54" s="23" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E54" s="23" t="s">
         <v>511</v>
@@ -6506,18 +6517,18 @@
         <v>500</v>
       </c>
       <c r="G54" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H54" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I54" s="23">
+        <v>554</v>
+      </c>
+      <c r="I54" s="34">
         <v>2.1</v>
       </c>
-      <c r="J54" s="23">
+      <c r="J54" s="34">
         <v>2</v>
       </c>
-      <c r="K54" s="23">
+      <c r="K54" s="34">
         <v>1</v>
       </c>
       <c r="L54" s="23" t="s">
@@ -6550,7 +6561,7 @@
         <v>246</v>
       </c>
       <c r="D55" s="23" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E55" s="23" t="s">
         <v>511</v>
@@ -6559,18 +6570,18 @@
         <v>500</v>
       </c>
       <c r="G55" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H55" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I55" s="23">
+        <v>554</v>
+      </c>
+      <c r="I55" s="34">
         <v>2.1</v>
       </c>
-      <c r="J55" s="23">
+      <c r="J55" s="34">
         <v>2</v>
       </c>
-      <c r="K55" s="23">
+      <c r="K55" s="34">
         <v>1</v>
       </c>
       <c r="L55" s="23" t="s">
@@ -6605,7 +6616,7 @@
         <v>246</v>
       </c>
       <c r="D56" s="23" t="s">
-        <v>596</v>
+        <v>592</v>
       </c>
       <c r="E56" s="23" t="s">
         <v>511</v>
@@ -6614,18 +6625,18 @@
         <v>500</v>
       </c>
       <c r="G56" s="23" t="s">
-        <v>584</v>
+        <v>580</v>
       </c>
       <c r="H56" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I56" s="23">
+        <v>554</v>
+      </c>
+      <c r="I56" s="34">
         <v>2.1</v>
       </c>
-      <c r="J56" s="23">
+      <c r="J56" s="34">
         <v>2</v>
       </c>
-      <c r="K56" s="23">
+      <c r="K56" s="34">
         <v>1</v>
       </c>
       <c r="L56" s="23" t="s">
@@ -6658,7 +6669,7 @@
         <v>246</v>
       </c>
       <c r="D57" s="23" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="E57" s="23" t="s">
         <v>506</v>
@@ -6667,18 +6678,18 @@
         <v>501</v>
       </c>
       <c r="G57" s="27" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H57" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I57" s="23">
+        <v>554</v>
+      </c>
+      <c r="I57" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J57" s="23">
+      <c r="J57" s="34">
         <v>2</v>
       </c>
-      <c r="K57" s="23">
+      <c r="K57" s="34">
         <v>2</v>
       </c>
       <c r="L57" s="23" t="s">
@@ -6713,7 +6724,7 @@
         <v>246</v>
       </c>
       <c r="D58" s="23" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="E58" s="23" t="s">
         <v>506</v>
@@ -6722,18 +6733,18 @@
         <v>501</v>
       </c>
       <c r="G58" s="23" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H58" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I58" s="23">
+        <v>554</v>
+      </c>
+      <c r="I58" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J58" s="23">
+      <c r="J58" s="34">
         <v>2</v>
       </c>
-      <c r="K58" s="23">
+      <c r="K58" s="34">
         <v>2</v>
       </c>
       <c r="L58" s="23" t="s">
@@ -6770,7 +6781,7 @@
         <v>246</v>
       </c>
       <c r="D59" s="23" t="s">
-        <v>597</v>
+        <v>593</v>
       </c>
       <c r="E59" s="26" t="s">
         <v>506</v>
@@ -6779,18 +6790,18 @@
         <v>501</v>
       </c>
       <c r="G59" s="26" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H59" s="26" t="s">
-        <v>556</v>
-      </c>
-      <c r="I59" s="26">
+        <v>554</v>
+      </c>
+      <c r="I59" s="39">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J59" s="26">
+      <c r="J59" s="39">
         <v>2</v>
       </c>
-      <c r="K59" s="26">
+      <c r="K59" s="39">
         <v>2</v>
       </c>
       <c r="L59" s="26" t="s">
@@ -6825,7 +6836,7 @@
         <v>246</v>
       </c>
       <c r="D60" s="23" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E60" s="23" t="s">
         <v>511</v>
@@ -6834,18 +6845,18 @@
         <v>500</v>
       </c>
       <c r="G60" s="23" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H60" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I60" s="23">
+        <v>554</v>
+      </c>
+      <c r="I60" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J60" s="23">
+      <c r="J60" s="34">
         <v>2</v>
       </c>
-      <c r="K60" s="23">
+      <c r="K60" s="34">
         <v>2</v>
       </c>
       <c r="L60" s="23" t="s">
@@ -6878,7 +6889,7 @@
         <v>246</v>
       </c>
       <c r="D61" s="23" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E61" s="23" t="s">
         <v>511</v>
@@ -6887,18 +6898,18 @@
         <v>500</v>
       </c>
       <c r="G61" s="23" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H61" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I61" s="23">
+        <v>554</v>
+      </c>
+      <c r="I61" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J61" s="23">
+      <c r="J61" s="34">
         <v>2</v>
       </c>
-      <c r="K61" s="23">
+      <c r="K61" s="34">
         <v>2</v>
       </c>
       <c r="L61" s="23" t="s">
@@ -6931,7 +6942,7 @@
         <v>246</v>
       </c>
       <c r="D62" s="23" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E62" s="23" t="s">
         <v>511</v>
@@ -6940,18 +6951,18 @@
         <v>500</v>
       </c>
       <c r="G62" s="23" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H62" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I62" s="23">
+        <v>554</v>
+      </c>
+      <c r="I62" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J62" s="23">
+      <c r="J62" s="34">
         <v>2</v>
       </c>
-      <c r="K62" s="23">
+      <c r="K62" s="34">
         <v>2</v>
       </c>
       <c r="L62" s="23" t="s">
@@ -6984,7 +6995,7 @@
         <v>246</v>
       </c>
       <c r="D63" s="23" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E63" s="23" t="s">
         <v>511</v>
@@ -6993,18 +7004,18 @@
         <v>500</v>
       </c>
       <c r="G63" s="23" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H63" s="23" t="s">
-        <v>556</v>
-      </c>
-      <c r="I63" s="23">
+        <v>554</v>
+      </c>
+      <c r="I63" s="34">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J63" s="23">
+      <c r="J63" s="34">
         <v>2</v>
       </c>
-      <c r="K63" s="23">
+      <c r="K63" s="34">
         <v>2</v>
       </c>
       <c r="L63" s="23" t="s">
@@ -7039,7 +7050,7 @@
         <v>246</v>
       </c>
       <c r="D64" s="23" t="s">
-        <v>598</v>
+        <v>594</v>
       </c>
       <c r="E64" s="26" t="s">
         <v>511</v>
@@ -7048,18 +7059,18 @@
         <v>500</v>
       </c>
       <c r="G64" s="26" t="s">
-        <v>585</v>
+        <v>581</v>
       </c>
       <c r="H64" s="26" t="s">
-        <v>556</v>
-      </c>
-      <c r="I64" s="26">
+        <v>554</v>
+      </c>
+      <c r="I64" s="39">
         <v>2.2000000000000002</v>
       </c>
-      <c r="J64" s="26">
+      <c r="J64" s="39">
         <v>2</v>
       </c>
-      <c r="K64" s="26">
+      <c r="K64" s="39">
         <v>2</v>
       </c>
       <c r="L64" s="26" t="s">
@@ -7094,7 +7105,7 @@
         <v>246</v>
       </c>
       <c r="D65" s="23" t="s">
-        <v>599</v>
+        <v>595</v>
       </c>
       <c r="E65" s="26" t="s">
         <v>502</v>
@@ -7103,18 +7114,18 @@
         <v>501</v>
       </c>
       <c r="G65" s="26" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="H65" s="26" t="s">
-        <v>557</v>
-      </c>
-      <c r="I65" s="26">
+        <v>555</v>
+      </c>
+      <c r="I65" s="39">
         <v>3</v>
       </c>
-      <c r="J65" s="26">
+      <c r="J65" s="39">
         <v>3</v>
       </c>
-      <c r="K65" s="26"/>
+      <c r="K65" s="39"/>
       <c r="L65" s="26" t="s">
         <v>232</v>
       </c>
@@ -7147,7 +7158,7 @@
         <v>246</v>
       </c>
       <c r="D66" s="23" t="s">
-        <v>600</v>
+        <v>596</v>
       </c>
       <c r="E66" s="23" t="s">
         <v>531</v>
@@ -7156,18 +7167,18 @@
         <v>500</v>
       </c>
       <c r="G66" s="23" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="H66" s="23" t="s">
-        <v>557</v>
-      </c>
-      <c r="I66" s="23">
+        <v>555</v>
+      </c>
+      <c r="I66" s="34">
         <v>3</v>
       </c>
-      <c r="J66" s="23">
+      <c r="J66" s="34">
         <v>3</v>
       </c>
-      <c r="K66" s="23"/>
+      <c r="K66" s="34"/>
       <c r="L66" s="23" t="s">
         <v>232</v>
       </c>
@@ -7200,7 +7211,7 @@
         <v>246</v>
       </c>
       <c r="D67" s="23" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="E67" s="26" t="s">
         <v>527</v>
@@ -7209,18 +7220,18 @@
         <v>501</v>
       </c>
       <c r="G67" s="26" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H67" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="I67" s="26">
+        <v>556</v>
+      </c>
+      <c r="I67" s="39">
         <v>4</v>
       </c>
-      <c r="J67" s="26">
+      <c r="J67" s="39">
         <v>4</v>
       </c>
-      <c r="K67" s="26"/>
+      <c r="K67" s="39"/>
       <c r="L67" s="26" t="s">
         <v>433</v>
       </c>
@@ -7251,7 +7262,7 @@
         <v>246</v>
       </c>
       <c r="D68" s="23" t="s">
-        <v>601</v>
+        <v>597</v>
       </c>
       <c r="E68" s="26" t="s">
         <v>527</v>
@@ -7260,18 +7271,18 @@
         <v>501</v>
       </c>
       <c r="G68" s="26" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H68" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="I68" s="26">
+        <v>556</v>
+      </c>
+      <c r="I68" s="39">
         <v>4</v>
       </c>
-      <c r="J68" s="26">
+      <c r="J68" s="39">
         <v>4</v>
       </c>
-      <c r="K68" s="26"/>
+      <c r="K68" s="39"/>
       <c r="L68" s="26" t="s">
         <v>229</v>
       </c>
@@ -7304,7 +7315,7 @@
         <v>246</v>
       </c>
       <c r="D69" s="23" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="E69" s="26" t="s">
         <v>528</v>
@@ -7313,18 +7324,18 @@
         <v>500</v>
       </c>
       <c r="G69" s="26" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H69" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="I69" s="26">
+        <v>556</v>
+      </c>
+      <c r="I69" s="39">
         <v>4</v>
       </c>
-      <c r="J69" s="26">
+      <c r="J69" s="39">
         <v>4</v>
       </c>
-      <c r="K69" s="26"/>
+      <c r="K69" s="39"/>
       <c r="L69" s="26" t="s">
         <v>433</v>
       </c>
@@ -7355,7 +7366,7 @@
         <v>246</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="E70" s="26" t="s">
         <v>528</v>
@@ -7364,18 +7375,18 @@
         <v>500</v>
       </c>
       <c r="G70" s="26" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H70" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="I70" s="26">
+        <v>556</v>
+      </c>
+      <c r="I70" s="39">
         <v>4</v>
       </c>
-      <c r="J70" s="26">
+      <c r="J70" s="39">
         <v>4</v>
       </c>
-      <c r="K70" s="26"/>
+      <c r="K70" s="39"/>
       <c r="L70" s="26" t="s">
         <v>231</v>
       </c>
@@ -7406,7 +7417,7 @@
         <v>246</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>602</v>
+        <v>598</v>
       </c>
       <c r="E71" s="26" t="s">
         <v>528</v>
@@ -7415,18 +7426,18 @@
         <v>500</v>
       </c>
       <c r="G71" s="26" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="H71" s="26" t="s">
-        <v>558</v>
-      </c>
-      <c r="I71" s="26">
+        <v>556</v>
+      </c>
+      <c r="I71" s="39">
         <v>4</v>
       </c>
-      <c r="J71" s="26">
+      <c r="J71" s="39">
         <v>4</v>
       </c>
-      <c r="K71" s="26"/>
+      <c r="K71" s="39"/>
       <c r="L71" s="26" t="s">
         <v>229</v>
       </c>
@@ -7457,7 +7468,7 @@
         <v>246</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>603</v>
+        <v>599</v>
       </c>
       <c r="E72" s="26" t="s">
         <v>530</v>
@@ -7466,18 +7477,18 @@
         <v>501</v>
       </c>
       <c r="G72" s="26" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="H72" s="26" t="s">
         <v>524</v>
       </c>
-      <c r="I72" s="26">
+      <c r="I72" s="39">
         <v>5</v>
       </c>
-      <c r="J72" s="26">
+      <c r="J72" s="39">
         <v>5</v>
       </c>
-      <c r="K72" s="26"/>
+      <c r="K72" s="39"/>
       <c r="L72" s="26" t="s">
         <v>523</v>
       </c>
@@ -7508,7 +7519,7 @@
         <v>246</v>
       </c>
       <c r="D73" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E73" s="27" t="s">
         <v>533</v>
@@ -7517,18 +7528,18 @@
         <v>500</v>
       </c>
       <c r="G73" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H73" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="I73" s="27">
+      <c r="I73" s="40">
         <v>6.1</v>
       </c>
-      <c r="J73" s="27">
+      <c r="J73" s="40">
         <v>6</v>
       </c>
-      <c r="K73" s="27">
+      <c r="K73" s="40">
         <v>1</v>
       </c>
       <c r="L73" s="23" t="s">
@@ -7561,7 +7572,7 @@
         <v>246</v>
       </c>
       <c r="D74" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E74" s="27" t="s">
         <v>533</v>
@@ -7570,18 +7581,18 @@
         <v>500</v>
       </c>
       <c r="G74" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H74" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="I74" s="27">
+      <c r="I74" s="40">
         <v>6.1</v>
       </c>
-      <c r="J74" s="27">
+      <c r="J74" s="40">
         <v>6</v>
       </c>
-      <c r="K74" s="27">
+      <c r="K74" s="40">
         <v>1</v>
       </c>
       <c r="L74" s="23" t="s">
@@ -7614,7 +7625,7 @@
         <v>246</v>
       </c>
       <c r="D75" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E75" s="23" t="s">
         <v>533</v>
@@ -7623,18 +7634,18 @@
         <v>500</v>
       </c>
       <c r="G75" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H75" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I75" s="23">
+      <c r="I75" s="34">
         <v>6.1</v>
       </c>
-      <c r="J75" s="27">
+      <c r="J75" s="40">
         <v>6</v>
       </c>
-      <c r="K75" s="23">
+      <c r="K75" s="34">
         <v>1</v>
       </c>
       <c r="L75" s="23" t="s">
@@ -7669,7 +7680,7 @@
         <v>246</v>
       </c>
       <c r="D76" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E76" s="23" t="s">
         <v>533</v>
@@ -7678,18 +7689,18 @@
         <v>500</v>
       </c>
       <c r="G76" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H76" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I76" s="23">
+      <c r="I76" s="34">
         <v>6.1</v>
       </c>
-      <c r="J76" s="27">
+      <c r="J76" s="40">
         <v>6</v>
       </c>
-      <c r="K76" s="23">
+      <c r="K76" s="34">
         <v>1</v>
       </c>
       <c r="L76" s="23" t="s">
@@ -7724,7 +7735,7 @@
         <v>246</v>
       </c>
       <c r="D77" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E77" s="23" t="s">
         <v>533</v>
@@ -7733,18 +7744,18 @@
         <v>500</v>
       </c>
       <c r="G77" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H77" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I77" s="23">
+      <c r="I77" s="34">
         <v>6.1</v>
       </c>
-      <c r="J77" s="27">
+      <c r="J77" s="40">
         <v>6</v>
       </c>
-      <c r="K77" s="23">
+      <c r="K77" s="34">
         <v>1</v>
       </c>
       <c r="L77" s="23" t="s">
@@ -7777,7 +7788,7 @@
         <v>246</v>
       </c>
       <c r="D78" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E78" s="23" t="s">
         <v>533</v>
@@ -7786,18 +7797,18 @@
         <v>500</v>
       </c>
       <c r="G78" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H78" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I78" s="23">
+      <c r="I78" s="34">
         <v>6.1</v>
       </c>
-      <c r="J78" s="27">
+      <c r="J78" s="40">
         <v>6</v>
       </c>
-      <c r="K78" s="23">
+      <c r="K78" s="34">
         <v>1</v>
       </c>
       <c r="L78" s="23" t="s">
@@ -7830,7 +7841,7 @@
         <v>246</v>
       </c>
       <c r="D79" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E79" s="23" t="s">
         <v>533</v>
@@ -7839,18 +7850,18 @@
         <v>500</v>
       </c>
       <c r="G79" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H79" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I79" s="23">
+      <c r="I79" s="34">
         <v>6.1</v>
       </c>
-      <c r="J79" s="27">
+      <c r="J79" s="40">
         <v>6</v>
       </c>
-      <c r="K79" s="23">
+      <c r="K79" s="34">
         <v>1</v>
       </c>
       <c r="L79" s="23" t="s">
@@ -7883,7 +7894,7 @@
         <v>246</v>
       </c>
       <c r="D80" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E80" s="23" t="s">
         <v>533</v>
@@ -7892,18 +7903,18 @@
         <v>500</v>
       </c>
       <c r="G80" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H80" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I80" s="23">
+      <c r="I80" s="34">
         <v>6.1</v>
       </c>
-      <c r="J80" s="27">
+      <c r="J80" s="40">
         <v>6</v>
       </c>
-      <c r="K80" s="23">
+      <c r="K80" s="34">
         <v>1</v>
       </c>
       <c r="L80" s="23" t="s">
@@ -7938,7 +7949,7 @@
         <v>246</v>
       </c>
       <c r="D81" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E81" s="27" t="s">
         <v>533</v>
@@ -7947,18 +7958,18 @@
         <v>500</v>
       </c>
       <c r="G81" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H81" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="I81" s="27">
+      <c r="I81" s="40">
         <v>6.1</v>
       </c>
-      <c r="J81" s="27">
+      <c r="J81" s="40">
         <v>6</v>
       </c>
-      <c r="K81" s="27">
+      <c r="K81" s="40">
         <v>1</v>
       </c>
       <c r="L81" s="23" t="s">
@@ -7993,7 +8004,7 @@
         <v>246</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E82" s="27" t="s">
         <v>533</v>
@@ -8002,18 +8013,18 @@
         <v>500</v>
       </c>
       <c r="G82" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H82" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="I82" s="27">
+      <c r="I82" s="40">
         <v>6.1</v>
       </c>
-      <c r="J82" s="27">
+      <c r="J82" s="40">
         <v>6</v>
       </c>
-      <c r="K82" s="27">
+      <c r="K82" s="40">
         <v>1</v>
       </c>
       <c r="L82" s="23" t="s">
@@ -8048,7 +8059,7 @@
         <v>246</v>
       </c>
       <c r="D83" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E83" s="27" t="s">
         <v>533</v>
@@ -8057,18 +8068,18 @@
         <v>500</v>
       </c>
       <c r="G83" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H83" s="27" t="s">
         <v>59</v>
       </c>
-      <c r="I83" s="27">
+      <c r="I83" s="40">
         <v>6.1</v>
       </c>
-      <c r="J83" s="27">
+      <c r="J83" s="40">
         <v>6</v>
       </c>
-      <c r="K83" s="27">
+      <c r="K83" s="40">
         <v>1</v>
       </c>
       <c r="L83" s="23" t="s">
@@ -8103,7 +8114,7 @@
         <v>246</v>
       </c>
       <c r="D84" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E84" s="23" t="s">
         <v>533</v>
@@ -8112,18 +8123,18 @@
         <v>500</v>
       </c>
       <c r="G84" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H84" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I84" s="23">
+      <c r="I84" s="34">
         <v>6.1</v>
       </c>
-      <c r="J84" s="27">
+      <c r="J84" s="40">
         <v>6</v>
       </c>
-      <c r="K84" s="23">
+      <c r="K84" s="34">
         <v>1</v>
       </c>
       <c r="L84" s="23" t="s">
@@ -8156,7 +8167,7 @@
         <v>246</v>
       </c>
       <c r="D85" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E85" s="23" t="s">
         <v>533</v>
@@ -8165,18 +8176,18 @@
         <v>500</v>
       </c>
       <c r="G85" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H85" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I85" s="23">
+      <c r="I85" s="34">
         <v>6.1</v>
       </c>
-      <c r="J85" s="27">
+      <c r="J85" s="40">
         <v>6</v>
       </c>
-      <c r="K85" s="23">
+      <c r="K85" s="34">
         <v>1</v>
       </c>
       <c r="L85" s="23" t="s">
@@ -8209,7 +8220,7 @@
         <v>246</v>
       </c>
       <c r="D86" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E86" s="23" t="s">
         <v>533</v>
@@ -8218,18 +8229,18 @@
         <v>500</v>
       </c>
       <c r="G86" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H86" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I86" s="23">
+      <c r="I86" s="34">
         <v>6.1</v>
       </c>
-      <c r="J86" s="27">
+      <c r="J86" s="40">
         <v>6</v>
       </c>
-      <c r="K86" s="23">
+      <c r="K86" s="34">
         <v>1</v>
       </c>
       <c r="L86" s="23" t="s">
@@ -8262,7 +8273,7 @@
         <v>246</v>
       </c>
       <c r="D87" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E87" s="23" t="s">
         <v>533</v>
@@ -8271,18 +8282,18 @@
         <v>500</v>
       </c>
       <c r="G87" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H87" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I87" s="23">
+      <c r="I87" s="34">
         <v>6.1</v>
       </c>
-      <c r="J87" s="27">
+      <c r="J87" s="40">
         <v>6</v>
       </c>
-      <c r="K87" s="23">
+      <c r="K87" s="34">
         <v>1</v>
       </c>
       <c r="L87" s="23" t="s">
@@ -8315,7 +8326,7 @@
         <v>246</v>
       </c>
       <c r="D88" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E88" s="23" t="s">
         <v>533</v>
@@ -8324,18 +8335,18 @@
         <v>500</v>
       </c>
       <c r="G88" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H88" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I88" s="23">
+      <c r="I88" s="34">
         <v>6.1</v>
       </c>
-      <c r="J88" s="27">
+      <c r="J88" s="40">
         <v>6</v>
       </c>
-      <c r="K88" s="23">
+      <c r="K88" s="34">
         <v>1</v>
       </c>
       <c r="L88" s="23" t="s">
@@ -8368,7 +8379,7 @@
         <v>246</v>
       </c>
       <c r="D89" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E89" s="23" t="s">
         <v>533</v>
@@ -8377,18 +8388,18 @@
         <v>500</v>
       </c>
       <c r="G89" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H89" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I89" s="23">
+      <c r="I89" s="34">
         <v>6.1</v>
       </c>
-      <c r="J89" s="27">
+      <c r="J89" s="40">
         <v>6</v>
       </c>
-      <c r="K89" s="23">
+      <c r="K89" s="34">
         <v>1</v>
       </c>
       <c r="L89" s="23" t="s">
@@ -8421,7 +8432,7 @@
         <v>246</v>
       </c>
       <c r="D90" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E90" s="23" t="s">
         <v>533</v>
@@ -8430,18 +8441,18 @@
         <v>500</v>
       </c>
       <c r="G90" s="23" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H90" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I90" s="23">
+      <c r="I90" s="34">
         <v>6.1</v>
       </c>
-      <c r="J90" s="27">
+      <c r="J90" s="40">
         <v>6</v>
       </c>
-      <c r="K90" s="23">
+      <c r="K90" s="34">
         <v>1</v>
       </c>
       <c r="L90" s="23" t="s">
@@ -8474,7 +8485,7 @@
         <v>246</v>
       </c>
       <c r="D91" s="23" t="s">
-        <v>604</v>
+        <v>600</v>
       </c>
       <c r="E91" s="23" t="s">
         <v>533</v>
@@ -8483,18 +8494,18 @@
         <v>500</v>
       </c>
       <c r="G91" s="31" t="s">
-        <v>586</v>
+        <v>582</v>
       </c>
       <c r="H91" s="32" t="s">
         <v>59</v>
       </c>
-      <c r="I91" s="33">
+      <c r="I91" s="41">
         <v>6.1</v>
       </c>
-      <c r="J91" s="27">
+      <c r="J91" s="40">
         <v>6</v>
       </c>
-      <c r="K91" s="23">
+      <c r="K91" s="34">
         <v>2</v>
       </c>
       <c r="L91" s="32" t="s">
@@ -8529,7 +8540,7 @@
         <v>246</v>
       </c>
       <c r="D92" s="23" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="E92" s="23" t="s">
         <v>534</v>
@@ -8538,18 +8549,18 @@
         <v>501</v>
       </c>
       <c r="G92" s="23" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="H92" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I92" s="23">
+      <c r="I92" s="34">
         <v>6.2</v>
       </c>
-      <c r="J92" s="27">
+      <c r="J92" s="40">
         <v>6</v>
       </c>
-      <c r="K92" s="23">
+      <c r="K92" s="34">
         <v>2</v>
       </c>
       <c r="L92" s="23" t="s">
@@ -8584,7 +8595,7 @@
         <v>246</v>
       </c>
       <c r="D93" s="23" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="E93" s="23" t="s">
         <v>534</v>
@@ -8593,18 +8604,18 @@
         <v>501</v>
       </c>
       <c r="G93" s="23" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="H93" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I93" s="23">
+      <c r="I93" s="34">
         <v>6.2</v>
       </c>
-      <c r="J93" s="27">
+      <c r="J93" s="40">
         <v>6</v>
       </c>
-      <c r="K93" s="23">
+      <c r="K93" s="34">
         <v>2</v>
       </c>
       <c r="L93" s="23" t="s">
@@ -8639,7 +8650,7 @@
         <v>246</v>
       </c>
       <c r="D94" s="23" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="E94" s="23" t="s">
         <v>534</v>
@@ -8648,18 +8659,18 @@
         <v>501</v>
       </c>
       <c r="G94" s="23" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="H94" s="23" t="s">
         <v>59</v>
       </c>
-      <c r="I94" s="23">
+      <c r="I94" s="34">
         <v>6.2</v>
       </c>
-      <c r="J94" s="27">
+      <c r="J94" s="40">
         <v>6</v>
       </c>
-      <c r="K94" s="23">
+      <c r="K94" s="34">
         <v>2</v>
       </c>
       <c r="L94" s="23" t="s">
@@ -8694,7 +8705,7 @@
         <v>246</v>
       </c>
       <c r="D95" s="23" t="s">
-        <v>605</v>
+        <v>601</v>
       </c>
       <c r="E95" s="26" t="s">
         <v>534</v>
@@ -8703,18 +8714,18 @@
         <v>501</v>
       </c>
       <c r="G95" s="26" t="s">
-        <v>587</v>
+        <v>583</v>
       </c>
       <c r="H95" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="I95" s="26">
+      <c r="I95" s="39">
         <v>6.2</v>
       </c>
-      <c r="J95" s="27">
+      <c r="J95" s="40">
         <v>6</v>
       </c>
-      <c r="K95" s="26">
+      <c r="K95" s="39">
         <v>2</v>
       </c>
       <c r="L95" s="26" t="s">
@@ -8749,7 +8760,7 @@
         <v>246</v>
       </c>
       <c r="D96" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E96" s="23" t="s">
         <v>540</v>
@@ -8758,18 +8769,18 @@
         <v>500</v>
       </c>
       <c r="G96" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H96" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I96" s="23">
+        <v>557</v>
+      </c>
+      <c r="I96" s="34">
         <v>7</v>
       </c>
-      <c r="J96" s="23">
+      <c r="J96" s="34">
         <v>7</v>
       </c>
-      <c r="K96" s="23"/>
+      <c r="K96" s="34"/>
       <c r="L96" s="23" t="s">
         <v>239</v>
       </c>
@@ -8800,7 +8811,7 @@
         <v>246</v>
       </c>
       <c r="D97" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E97" s="23" t="s">
         <v>540</v>
@@ -8809,18 +8820,18 @@
         <v>500</v>
       </c>
       <c r="G97" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H97" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I97" s="23">
+        <v>557</v>
+      </c>
+      <c r="I97" s="34">
         <v>7</v>
       </c>
-      <c r="J97" s="23">
+      <c r="J97" s="34">
         <v>7</v>
       </c>
-      <c r="K97" s="23"/>
+      <c r="K97" s="34"/>
       <c r="L97" s="23" t="s">
         <v>242</v>
       </c>
@@ -8853,7 +8864,7 @@
         <v>246</v>
       </c>
       <c r="D98" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E98" s="23" t="s">
         <v>540</v>
@@ -8862,18 +8873,18 @@
         <v>500</v>
       </c>
       <c r="G98" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H98" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I98" s="23">
+        <v>557</v>
+      </c>
+      <c r="I98" s="34">
         <v>7</v>
       </c>
-      <c r="J98" s="23">
+      <c r="J98" s="34">
         <v>7</v>
       </c>
-      <c r="K98" s="23"/>
+      <c r="K98" s="34"/>
       <c r="L98" s="23" t="s">
         <v>364</v>
       </c>
@@ -8906,7 +8917,7 @@
         <v>246</v>
       </c>
       <c r="D99" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E99" s="23" t="s">
         <v>540</v>
@@ -8915,18 +8926,18 @@
         <v>500</v>
       </c>
       <c r="G99" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H99" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I99" s="23">
+        <v>557</v>
+      </c>
+      <c r="I99" s="34">
         <v>7</v>
       </c>
-      <c r="J99" s="23">
+      <c r="J99" s="34">
         <v>7</v>
       </c>
-      <c r="K99" s="23"/>
+      <c r="K99" s="34"/>
       <c r="L99" s="23" t="s">
         <v>243</v>
       </c>
@@ -8959,7 +8970,7 @@
         <v>246</v>
       </c>
       <c r="D100" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E100" s="23" t="s">
         <v>540</v>
@@ -8968,18 +8979,18 @@
         <v>500</v>
       </c>
       <c r="G100" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H100" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I100" s="23">
+        <v>557</v>
+      </c>
+      <c r="I100" s="34">
         <v>7</v>
       </c>
-      <c r="J100" s="23">
+      <c r="J100" s="34">
         <v>7</v>
       </c>
-      <c r="K100" s="23"/>
+      <c r="K100" s="34"/>
       <c r="L100" s="23" t="s">
         <v>220</v>
       </c>
@@ -9012,7 +9023,7 @@
         <v>246</v>
       </c>
       <c r="D101" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E101" s="23" t="s">
         <v>540</v>
@@ -9021,18 +9032,18 @@
         <v>500</v>
       </c>
       <c r="G101" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H101" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I101" s="23">
+        <v>557</v>
+      </c>
+      <c r="I101" s="34">
         <v>7</v>
       </c>
-      <c r="J101" s="23">
+      <c r="J101" s="34">
         <v>7</v>
       </c>
-      <c r="K101" s="23"/>
+      <c r="K101" s="34"/>
       <c r="L101" s="23" t="s">
         <v>220</v>
       </c>
@@ -9063,7 +9074,7 @@
         <v>246</v>
       </c>
       <c r="D102" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E102" s="23" t="s">
         <v>540</v>
@@ -9072,18 +9083,18 @@
         <v>500</v>
       </c>
       <c r="G102" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H102" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I102" s="23">
+        <v>557</v>
+      </c>
+      <c r="I102" s="34">
         <v>7</v>
       </c>
-      <c r="J102" s="23">
+      <c r="J102" s="34">
         <v>7</v>
       </c>
-      <c r="K102" s="23"/>
+      <c r="K102" s="34"/>
       <c r="L102" s="23" t="s">
         <v>288</v>
       </c>
@@ -9116,7 +9127,7 @@
         <v>246</v>
       </c>
       <c r="D103" s="23" t="s">
-        <v>606</v>
+        <v>602</v>
       </c>
       <c r="E103" s="23" t="s">
         <v>540</v>
@@ -9125,18 +9136,18 @@
         <v>500</v>
       </c>
       <c r="G103" s="23" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="H103" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I103" s="23">
+        <v>557</v>
+      </c>
+      <c r="I103" s="34">
         <v>7</v>
       </c>
-      <c r="J103" s="23">
+      <c r="J103" s="34">
         <v>7</v>
       </c>
-      <c r="K103" s="23"/>
+      <c r="K103" s="34"/>
       <c r="L103" s="23" t="s">
         <v>288</v>
       </c>
@@ -9167,7 +9178,7 @@
         <v>246</v>
       </c>
       <c r="D104" s="23" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="E104" s="23" t="s">
         <v>541</v>
@@ -9176,18 +9187,18 @@
         <v>500</v>
       </c>
       <c r="G104" s="23" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H104" s="23" t="s">
-        <v>560</v>
-      </c>
-      <c r="I104" s="23">
+        <v>558</v>
+      </c>
+      <c r="I104" s="34">
         <v>8</v>
       </c>
-      <c r="J104" s="23">
+      <c r="J104" s="34">
         <v>8</v>
       </c>
-      <c r="K104" s="23"/>
+      <c r="K104" s="34"/>
       <c r="L104" s="23" t="s">
         <v>225</v>
       </c>
@@ -9220,7 +9231,7 @@
         <v>246</v>
       </c>
       <c r="D105" s="23" t="s">
-        <v>607</v>
+        <v>603</v>
       </c>
       <c r="E105" s="23" t="s">
         <v>541</v>
@@ -9229,18 +9240,18 @@
         <v>500</v>
       </c>
       <c r="G105" s="23" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="H105" s="23" t="s">
-        <v>560</v>
-      </c>
-      <c r="I105" s="23">
+        <v>558</v>
+      </c>
+      <c r="I105" s="34">
         <v>8</v>
       </c>
-      <c r="J105" s="23">
+      <c r="J105" s="34">
         <v>8</v>
       </c>
-      <c r="K105" s="23"/>
+      <c r="K105" s="34"/>
       <c r="L105" s="23" t="s">
         <v>225</v>
       </c>
@@ -9271,7 +9282,7 @@
         <v>246</v>
       </c>
       <c r="D106" s="23" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="E106" s="23" t="s">
         <v>538</v>
@@ -9280,18 +9291,18 @@
         <v>500</v>
       </c>
       <c r="G106" s="23" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H106" s="23" t="s">
-        <v>561</v>
-      </c>
-      <c r="I106" s="23">
+        <v>559</v>
+      </c>
+      <c r="I106" s="34">
         <v>9</v>
       </c>
-      <c r="J106" s="23">
+      <c r="J106" s="34">
         <v>9</v>
       </c>
-      <c r="K106" s="23"/>
+      <c r="K106" s="34"/>
       <c r="L106" s="23" t="s">
         <v>238</v>
       </c>
@@ -9324,7 +9335,7 @@
         <v>246</v>
       </c>
       <c r="D107" s="23" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="E107" s="23" t="s">
         <v>538</v>
@@ -9333,18 +9344,18 @@
         <v>500</v>
       </c>
       <c r="G107" s="23" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H107" s="23" t="s">
-        <v>561</v>
-      </c>
-      <c r="I107" s="23">
+        <v>559</v>
+      </c>
+      <c r="I107" s="34">
         <v>9</v>
       </c>
-      <c r="J107" s="23">
+      <c r="J107" s="34">
         <v>9</v>
       </c>
-      <c r="K107" s="23"/>
+      <c r="K107" s="34"/>
       <c r="L107" s="23" t="s">
         <v>223</v>
       </c>
@@ -9377,7 +9388,7 @@
         <v>246</v>
       </c>
       <c r="D108" s="23" t="s">
-        <v>608</v>
+        <v>604</v>
       </c>
       <c r="E108" s="23" t="s">
         <v>538</v>
@@ -9386,18 +9397,18 @@
         <v>500</v>
       </c>
       <c r="G108" s="23" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="H108" s="23" t="s">
-        <v>561</v>
-      </c>
-      <c r="I108" s="23">
+        <v>559</v>
+      </c>
+      <c r="I108" s="34">
         <v>9</v>
       </c>
-      <c r="J108" s="23">
+      <c r="J108" s="34">
         <v>9</v>
       </c>
-      <c r="K108" s="23"/>
+      <c r="K108" s="34"/>
       <c r="L108" s="23" t="s">
         <v>152</v>
       </c>
@@ -9428,7 +9439,7 @@
         <v>246</v>
       </c>
       <c r="D109" s="23" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="E109" s="23" t="s">
         <v>535</v>
@@ -9437,18 +9448,18 @@
         <v>500</v>
       </c>
       <c r="G109" s="23" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H109" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I109" s="23">
+        <v>560</v>
+      </c>
+      <c r="I109" s="34">
         <v>10</v>
       </c>
-      <c r="J109" s="23">
+      <c r="J109" s="34">
         <v>10</v>
       </c>
-      <c r="K109" s="23"/>
+      <c r="K109" s="34"/>
       <c r="L109" s="23" t="s">
         <v>219</v>
       </c>
@@ -9483,7 +9494,7 @@
         <v>246</v>
       </c>
       <c r="D110" s="23" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="E110" s="23" t="s">
         <v>535</v>
@@ -9492,18 +9503,18 @@
         <v>500</v>
       </c>
       <c r="G110" s="23" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H110" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I110" s="23">
+        <v>560</v>
+      </c>
+      <c r="I110" s="34">
         <v>10</v>
       </c>
-      <c r="J110" s="23">
+      <c r="J110" s="34">
         <v>10</v>
       </c>
-      <c r="K110" s="23"/>
+      <c r="K110" s="34"/>
       <c r="L110" s="23" t="s">
         <v>356</v>
       </c>
@@ -9534,7 +9545,7 @@
         <v>246</v>
       </c>
       <c r="D111" s="23" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="E111" s="23" t="s">
         <v>535</v>
@@ -9543,18 +9554,18 @@
         <v>500</v>
       </c>
       <c r="G111" s="23" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H111" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I111" s="23">
+        <v>560</v>
+      </c>
+      <c r="I111" s="34">
         <v>10</v>
       </c>
-      <c r="J111" s="23">
+      <c r="J111" s="34">
         <v>10</v>
       </c>
-      <c r="K111" s="23"/>
+      <c r="K111" s="34"/>
       <c r="L111" s="23" t="s">
         <v>462</v>
       </c>
@@ -9585,7 +9596,7 @@
         <v>246</v>
       </c>
       <c r="D112" s="23" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="E112" s="23" t="s">
         <v>535</v>
@@ -9594,18 +9605,18 @@
         <v>500</v>
       </c>
       <c r="G112" s="23" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H112" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I112" s="23">
+        <v>560</v>
+      </c>
+      <c r="I112" s="34">
         <v>10</v>
       </c>
-      <c r="J112" s="23">
+      <c r="J112" s="34">
         <v>10</v>
       </c>
-      <c r="K112" s="23"/>
+      <c r="K112" s="34"/>
       <c r="L112" s="23" t="s">
         <v>460</v>
       </c>
@@ -9636,7 +9647,7 @@
         <v>246</v>
       </c>
       <c r="D113" s="23" t="s">
-        <v>609</v>
+        <v>605</v>
       </c>
       <c r="E113" s="23" t="s">
         <v>535</v>
@@ -9645,18 +9656,18 @@
         <v>500</v>
       </c>
       <c r="G113" s="23" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="H113" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I113" s="23">
+        <v>560</v>
+      </c>
+      <c r="I113" s="34">
         <v>10</v>
       </c>
-      <c r="J113" s="23">
+      <c r="J113" s="34">
         <v>10</v>
       </c>
-      <c r="K113" s="23"/>
+      <c r="K113" s="34"/>
       <c r="L113" s="23" t="s">
         <v>463</v>
       </c>
@@ -9687,7 +9698,7 @@
         <v>246</v>
       </c>
       <c r="D114" s="23" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="E114" s="23" t="s">
         <v>536</v>
@@ -9696,18 +9707,18 @@
         <v>501</v>
       </c>
       <c r="G114" s="23" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H114" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I114" s="23">
+        <v>560</v>
+      </c>
+      <c r="I114" s="34">
         <v>11</v>
       </c>
-      <c r="J114" s="23">
+      <c r="J114" s="34">
         <v>11</v>
       </c>
-      <c r="K114" s="23"/>
+      <c r="K114" s="34"/>
       <c r="L114" s="23" t="s">
         <v>219</v>
       </c>
@@ -9742,7 +9753,7 @@
         <v>246</v>
       </c>
       <c r="D115" s="23" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="E115" s="23" t="s">
         <v>536</v>
@@ -9751,18 +9762,18 @@
         <v>501</v>
       </c>
       <c r="G115" s="23" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H115" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I115" s="23">
+        <v>560</v>
+      </c>
+      <c r="I115" s="34">
         <v>11</v>
       </c>
-      <c r="J115" s="23">
+      <c r="J115" s="34">
         <v>11</v>
       </c>
-      <c r="K115" s="23"/>
+      <c r="K115" s="34"/>
       <c r="L115" s="23" t="s">
         <v>218</v>
       </c>
@@ -9795,7 +9806,7 @@
         <v>246</v>
       </c>
       <c r="D116" s="23" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="E116" s="23" t="s">
         <v>536</v>
@@ -9804,18 +9815,18 @@
         <v>501</v>
       </c>
       <c r="G116" s="23" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H116" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I116" s="23">
+        <v>560</v>
+      </c>
+      <c r="I116" s="34">
         <v>11</v>
       </c>
-      <c r="J116" s="23">
+      <c r="J116" s="34">
         <v>11</v>
       </c>
-      <c r="K116" s="23"/>
+      <c r="K116" s="34"/>
       <c r="L116" s="23" t="s">
         <v>307</v>
       </c>
@@ -9846,7 +9857,7 @@
         <v>246</v>
       </c>
       <c r="D117" s="23" t="s">
-        <v>610</v>
+        <v>606</v>
       </c>
       <c r="E117" s="23" t="s">
         <v>536</v>
@@ -9855,18 +9866,18 @@
         <v>501</v>
       </c>
       <c r="G117" s="27" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="H117" s="23" t="s">
-        <v>562</v>
-      </c>
-      <c r="I117" s="23">
+        <v>560</v>
+      </c>
+      <c r="I117" s="34">
         <v>11</v>
       </c>
-      <c r="J117" s="23">
+      <c r="J117" s="34">
         <v>11</v>
       </c>
-      <c r="K117" s="23"/>
+      <c r="K117" s="34"/>
       <c r="L117" s="23" t="s">
         <v>218</v>
       </c>
@@ -9897,7 +9908,7 @@
         <v>246</v>
       </c>
       <c r="D118" s="23" t="s">
-        <v>611</v>
+        <v>607</v>
       </c>
       <c r="E118" s="23" t="s">
         <v>505</v>
@@ -9906,18 +9917,18 @@
         <v>501</v>
       </c>
       <c r="G118" s="23" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="H118" s="23" t="s">
         <v>124</v>
       </c>
-      <c r="I118" s="23">
+      <c r="I118" s="34">
         <v>12</v>
       </c>
-      <c r="J118" s="23">
+      <c r="J118" s="34">
         <v>12</v>
       </c>
-      <c r="K118" s="23"/>
+      <c r="K118" s="34"/>
       <c r="L118" s="23" t="s">
         <v>226</v>
       </c>
@@ -9950,7 +9961,7 @@
         <v>246</v>
       </c>
       <c r="D119" s="23" t="s">
-        <v>612</v>
+        <v>608</v>
       </c>
       <c r="E119" s="23" t="s">
         <v>532</v>
@@ -9959,18 +9970,18 @@
         <v>501</v>
       </c>
       <c r="G119" s="23" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="H119" s="23" t="s">
-        <v>560</v>
-      </c>
-      <c r="I119" s="23">
+        <v>558</v>
+      </c>
+      <c r="I119" s="34">
         <v>13</v>
       </c>
-      <c r="J119" s="23">
+      <c r="J119" s="34">
         <v>13</v>
       </c>
-      <c r="K119" s="23"/>
+      <c r="K119" s="34"/>
       <c r="L119" s="23" t="s">
         <v>225</v>
       </c>
@@ -10003,7 +10014,7 @@
         <v>246</v>
       </c>
       <c r="D120" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E120" s="24" t="s">
         <v>507</v>
@@ -10012,18 +10023,18 @@
         <v>501</v>
       </c>
       <c r="G120" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H120" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I120" s="24">
+      <c r="I120" s="42">
         <v>14</v>
       </c>
-      <c r="J120" s="23">
+      <c r="J120" s="34">
         <v>14</v>
       </c>
-      <c r="K120" s="24"/>
+      <c r="K120" s="42"/>
       <c r="L120" s="24" t="s">
         <v>357</v>
       </c>
@@ -10054,7 +10065,7 @@
         <v>246</v>
       </c>
       <c r="D121" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E121" s="24" t="s">
         <v>507</v>
@@ -10063,18 +10074,18 @@
         <v>501</v>
       </c>
       <c r="G121" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H121" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I121" s="24">
+      <c r="I121" s="42">
         <v>14</v>
       </c>
-      <c r="J121" s="23">
+      <c r="J121" s="34">
         <v>14</v>
       </c>
-      <c r="K121" s="24"/>
+      <c r="K121" s="42"/>
       <c r="L121" s="24" t="s">
         <v>304</v>
       </c>
@@ -10105,7 +10116,7 @@
         <v>246</v>
       </c>
       <c r="D122" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E122" s="24" t="s">
         <v>507</v>
@@ -10114,18 +10125,18 @@
         <v>501</v>
       </c>
       <c r="G122" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H122" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I122" s="24">
+      <c r="I122" s="42">
         <v>14</v>
       </c>
-      <c r="J122" s="23">
+      <c r="J122" s="34">
         <v>14</v>
       </c>
-      <c r="K122" s="24"/>
+      <c r="K122" s="42"/>
       <c r="L122" s="24" t="s">
         <v>359</v>
       </c>
@@ -10158,7 +10169,7 @@
         <v>246</v>
       </c>
       <c r="D123" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E123" s="24" t="s">
         <v>507</v>
@@ -10167,18 +10178,18 @@
         <v>501</v>
       </c>
       <c r="G123" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H123" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I123" s="24">
+      <c r="I123" s="42">
         <v>14</v>
       </c>
-      <c r="J123" s="23">
+      <c r="J123" s="34">
         <v>14</v>
       </c>
-      <c r="K123" s="24"/>
+      <c r="K123" s="42"/>
       <c r="L123" s="24" t="s">
         <v>218</v>
       </c>
@@ -10211,7 +10222,7 @@
         <v>246</v>
       </c>
       <c r="D124" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E124" s="24" t="s">
         <v>507</v>
@@ -10220,18 +10231,18 @@
         <v>501</v>
       </c>
       <c r="G124" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H124" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I124" s="24">
+      <c r="I124" s="42">
         <v>14</v>
       </c>
-      <c r="J124" s="23">
+      <c r="J124" s="34">
         <v>14</v>
       </c>
-      <c r="K124" s="24"/>
+      <c r="K124" s="42"/>
       <c r="L124" s="24" t="s">
         <v>225</v>
       </c>
@@ -10264,7 +10275,7 @@
         <v>246</v>
       </c>
       <c r="D125" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E125" s="24" t="s">
         <v>507</v>
@@ -10273,18 +10284,18 @@
         <v>501</v>
       </c>
       <c r="G125" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H125" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I125" s="24">
+      <c r="I125" s="42">
         <v>14</v>
       </c>
-      <c r="J125" s="23">
+      <c r="J125" s="34">
         <v>14</v>
       </c>
-      <c r="K125" s="24"/>
+      <c r="K125" s="42"/>
       <c r="L125" s="24" t="s">
         <v>219</v>
       </c>
@@ -10319,7 +10330,7 @@
         <v>246</v>
       </c>
       <c r="D126" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E126" s="24" t="s">
         <v>507</v>
@@ -10328,18 +10339,18 @@
         <v>501</v>
       </c>
       <c r="G126" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H126" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I126" s="24">
+      <c r="I126" s="42">
         <v>14</v>
       </c>
-      <c r="J126" s="23">
+      <c r="J126" s="34">
         <v>14</v>
       </c>
-      <c r="K126" s="24"/>
+      <c r="K126" s="42"/>
       <c r="L126" s="24" t="s">
         <v>7</v>
       </c>
@@ -10372,7 +10383,7 @@
         <v>246</v>
       </c>
       <c r="D127" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E127" s="24" t="s">
         <v>507</v>
@@ -10381,18 +10392,18 @@
         <v>501</v>
       </c>
       <c r="G127" s="27" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H127" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I127" s="24">
+      <c r="I127" s="42">
         <v>14</v>
       </c>
-      <c r="J127" s="23">
+      <c r="J127" s="34">
         <v>14</v>
       </c>
-      <c r="K127" s="24"/>
+      <c r="K127" s="42"/>
       <c r="L127" s="24" t="s">
         <v>238</v>
       </c>
@@ -10425,7 +10436,7 @@
         <v>246</v>
       </c>
       <c r="D128" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E128" s="24" t="s">
         <v>507</v>
@@ -10434,18 +10445,18 @@
         <v>501</v>
       </c>
       <c r="G128" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H128" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I128" s="24">
+      <c r="I128" s="42">
         <v>14</v>
       </c>
-      <c r="J128" s="23">
+      <c r="J128" s="34">
         <v>14</v>
       </c>
-      <c r="K128" s="24"/>
+      <c r="K128" s="42"/>
       <c r="L128" s="24" t="s">
         <v>226</v>
       </c>
@@ -10478,7 +10489,7 @@
         <v>246</v>
       </c>
       <c r="D129" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E129" s="24" t="s">
         <v>507</v>
@@ -10487,18 +10498,18 @@
         <v>501</v>
       </c>
       <c r="G129" s="23" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H129" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I129" s="24">
+      <c r="I129" s="42">
         <v>14</v>
       </c>
-      <c r="J129" s="23">
+      <c r="J129" s="34">
         <v>14</v>
       </c>
-      <c r="K129" s="24"/>
+      <c r="K129" s="42"/>
       <c r="L129" s="24" t="s">
         <v>236</v>
       </c>
@@ -10531,7 +10542,7 @@
         <v>246</v>
       </c>
       <c r="D130" s="23" t="s">
-        <v>613</v>
+        <v>609</v>
       </c>
       <c r="E130" s="24" t="s">
         <v>507</v>
@@ -10540,18 +10551,18 @@
         <v>501</v>
       </c>
       <c r="G130" s="27" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="H130" s="24" t="s">
         <v>491</v>
       </c>
-      <c r="I130" s="24">
+      <c r="I130" s="42">
         <v>14</v>
       </c>
-      <c r="J130" s="23">
+      <c r="J130" s="34">
         <v>14</v>
       </c>
-      <c r="K130" s="24"/>
+      <c r="K130" s="42"/>
       <c r="L130" s="24" t="s">
         <v>239</v>
       </c>
@@ -10582,7 +10593,7 @@
         <v>246</v>
       </c>
       <c r="D131" s="23" t="s">
-        <v>614</v>
+        <v>610</v>
       </c>
       <c r="E131" s="23" t="s">
         <v>508</v>
@@ -10591,18 +10602,18 @@
         <v>501</v>
       </c>
       <c r="G131" s="23" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="H131" s="23" t="s">
         <v>94</v>
       </c>
-      <c r="I131" s="23">
+      <c r="I131" s="34">
         <v>15</v>
       </c>
-      <c r="J131" s="23">
+      <c r="J131" s="34">
         <v>15</v>
       </c>
-      <c r="K131" s="23"/>
+      <c r="K131" s="34"/>
       <c r="L131" s="23" t="s">
         <v>214</v>
       </c>
@@ -10637,7 +10648,7 @@
         <v>246</v>
       </c>
       <c r="D132" s="23" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="E132" s="24" t="s">
         <v>544</v>
@@ -10646,18 +10657,18 @@
         <v>501</v>
       </c>
       <c r="G132" s="23" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="H132" s="24" t="s">
-        <v>563</v>
-      </c>
-      <c r="I132" s="24">
+        <v>561</v>
+      </c>
+      <c r="I132" s="42">
         <v>16</v>
       </c>
-      <c r="J132" s="23">
+      <c r="J132" s="34">
         <v>16</v>
       </c>
-      <c r="K132" s="24"/>
+      <c r="K132" s="42"/>
       <c r="L132" s="23" t="s">
         <v>285</v>
       </c>
@@ -10688,7 +10699,7 @@
         <v>246</v>
       </c>
       <c r="D133" s="23" t="s">
-        <v>615</v>
+        <v>611</v>
       </c>
       <c r="E133" s="24" t="s">
         <v>544</v>
@@ -10697,18 +10708,18 @@
         <v>501</v>
       </c>
       <c r="G133" s="23" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="H133" s="24" t="s">
-        <v>563</v>
-      </c>
-      <c r="I133" s="24">
+        <v>561</v>
+      </c>
+      <c r="I133" s="42">
         <v>16</v>
       </c>
-      <c r="J133" s="23">
+      <c r="J133" s="34">
         <v>16</v>
       </c>
-      <c r="K133" s="24"/>
+      <c r="K133" s="42"/>
       <c r="L133" s="23" t="s">
         <v>358</v>
       </c>
@@ -10739,7 +10750,7 @@
         <v>246</v>
       </c>
       <c r="D134" s="23" t="s">
-        <v>616</v>
+        <v>612</v>
       </c>
       <c r="E134" s="23" t="s">
         <v>542</v>
@@ -10748,18 +10759,18 @@
         <v>501</v>
       </c>
       <c r="G134" s="23" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H134" s="23" t="s">
-        <v>564</v>
-      </c>
-      <c r="I134" s="23">
+        <v>562</v>
+      </c>
+      <c r="I134" s="34">
         <v>16</v>
       </c>
-      <c r="J134" s="23">
+      <c r="J134" s="34">
         <v>16</v>
       </c>
-      <c r="K134" s="23"/>
+      <c r="K134" s="34"/>
       <c r="L134" s="23" t="s">
         <v>234</v>
       </c>
@@ -10792,7 +10803,7 @@
         <v>246</v>
       </c>
       <c r="D135" s="23" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="E135" s="24" t="s">
         <v>546</v>
@@ -10801,18 +10812,18 @@
         <v>501</v>
       </c>
       <c r="G135" s="23" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H135" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="I135" s="24">
+      <c r="I135" s="42">
         <v>16</v>
       </c>
-      <c r="J135" s="23">
+      <c r="J135" s="34">
         <v>16</v>
       </c>
-      <c r="K135" s="24"/>
+      <c r="K135" s="42"/>
       <c r="L135" s="23" t="s">
         <v>235</v>
       </c>
@@ -10847,7 +10858,7 @@
         <v>246</v>
       </c>
       <c r="D136" s="23" t="s">
-        <v>617</v>
+        <v>613</v>
       </c>
       <c r="E136" s="24" t="s">
         <v>546</v>
@@ -10856,18 +10867,18 @@
         <v>501</v>
       </c>
       <c r="G136" s="23" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="H136" s="24" t="s">
         <v>123</v>
       </c>
-      <c r="I136" s="24">
+      <c r="I136" s="42">
         <v>16</v>
       </c>
-      <c r="J136" s="23">
+      <c r="J136" s="34">
         <v>16</v>
       </c>
-      <c r="K136" s="24"/>
+      <c r="K136" s="42"/>
       <c r="L136" s="24" t="s">
         <v>235</v>
       </c>
@@ -10902,7 +10913,7 @@
         <v>246</v>
       </c>
       <c r="D137" s="23" t="s">
-        <v>618</v>
+        <v>614</v>
       </c>
       <c r="E137" s="23" t="s">
         <v>545</v>
@@ -10911,18 +10922,18 @@
         <v>500</v>
       </c>
       <c r="G137" s="23" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="H137" s="23" t="s">
-        <v>563</v>
-      </c>
-      <c r="I137" s="23">
+        <v>561</v>
+      </c>
+      <c r="I137" s="34">
         <v>16</v>
       </c>
-      <c r="J137" s="23">
+      <c r="J137" s="34">
         <v>16</v>
       </c>
-      <c r="K137" s="23"/>
+      <c r="K137" s="34"/>
       <c r="L137" s="23" t="s">
         <v>358</v>
       </c>
@@ -10953,7 +10964,7 @@
         <v>246</v>
       </c>
       <c r="D138" s="23" t="s">
-        <v>619</v>
+        <v>615</v>
       </c>
       <c r="E138" s="23" t="s">
         <v>543</v>
@@ -10962,18 +10973,18 @@
         <v>500</v>
       </c>
       <c r="G138" s="23" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="H138" s="23" t="s">
-        <v>564</v>
-      </c>
-      <c r="I138" s="23">
+        <v>562</v>
+      </c>
+      <c r="I138" s="34">
         <v>16</v>
       </c>
-      <c r="J138" s="23">
+      <c r="J138" s="34">
         <v>16</v>
       </c>
-      <c r="K138" s="23"/>
+      <c r="K138" s="34"/>
       <c r="L138" s="23" t="s">
         <v>240</v>
       </c>
@@ -11008,7 +11019,7 @@
         <v>246</v>
       </c>
       <c r="D139" s="23" t="s">
-        <v>622</v>
+        <v>618</v>
       </c>
       <c r="E139" s="23" t="s">
         <v>529</v>
@@ -11017,18 +11028,18 @@
         <v>500</v>
       </c>
       <c r="G139" s="23" t="s">
-        <v>588</v>
+        <v>584</v>
       </c>
       <c r="H139" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="I139" s="23" t="s">
-        <v>552</v>
-      </c>
-      <c r="J139" s="23" t="s">
-        <v>552</v>
-      </c>
-      <c r="K139" s="23"/>
+      <c r="I139" s="34" t="s">
+        <v>550</v>
+      </c>
+      <c r="J139" s="34" t="s">
+        <v>550</v>
+      </c>
+      <c r="K139" s="34"/>
       <c r="L139" s="23" t="s">
         <v>233</v>
       </c>
@@ -11061,7 +11072,7 @@
         <v>246</v>
       </c>
       <c r="D140" s="23" t="s">
-        <v>621</v>
+        <v>617</v>
       </c>
       <c r="E140" s="23" t="s">
         <v>539</v>
@@ -11070,18 +11081,18 @@
         <v>501</v>
       </c>
       <c r="G140" s="23" t="s">
-        <v>589</v>
+        <v>585</v>
       </c>
       <c r="H140" s="23" t="s">
-        <v>561</v>
-      </c>
-      <c r="I140" s="23" t="s">
-        <v>553</v>
-      </c>
-      <c r="J140" s="23" t="s">
-        <v>553</v>
-      </c>
-      <c r="K140" s="23"/>
+        <v>559</v>
+      </c>
+      <c r="I140" s="34" t="s">
+        <v>551</v>
+      </c>
+      <c r="J140" s="34" t="s">
+        <v>551</v>
+      </c>
+      <c r="K140" s="34"/>
       <c r="L140" s="23" t="s">
         <v>223</v>
       </c>
@@ -11114,7 +11125,7 @@
         <v>246</v>
       </c>
       <c r="D141" s="38" t="s">
-        <v>620</v>
+        <v>616</v>
       </c>
       <c r="E141" s="23" t="s">
         <v>537</v>
@@ -11123,18 +11134,18 @@
         <v>501</v>
       </c>
       <c r="G141" s="23" t="s">
-        <v>590</v>
+        <v>586</v>
       </c>
       <c r="H141" s="23" t="s">
-        <v>559</v>
-      </c>
-      <c r="I141" s="23" t="s">
-        <v>554</v>
-      </c>
-      <c r="J141" s="23" t="s">
-        <v>554</v>
-      </c>
-      <c r="K141" s="23"/>
+        <v>557</v>
+      </c>
+      <c r="I141" s="34" t="s">
+        <v>552</v>
+      </c>
+      <c r="J141" s="34" t="s">
+        <v>552</v>
+      </c>
+      <c r="K141" s="34"/>
       <c r="L141" s="23" t="s">
         <v>220</v>
       </c>

</xml_diff>